<commit_message>
Add EVIDENCE_MAP.md and update DOCUMENT_INDEX.xlsx with issue tags
</commit_message>
<xml_diff>
--- a/00_CASE_SUMMARY/DOCUMENT_INDEX.xlsx
+++ b/00_CASE_SUMMARY/DOCUMENT_INDEX.xlsx
@@ -4070,7 +4070,11 @@
           <t>PNG</t>
         </is>
       </c>
-      <c r="F78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
       <c r="G78" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -4081,10 +4085,14 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="I78" s="2" t="inlineStr"/>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>Text to Ford, no response - non-response pattern.</t>
+        </is>
+      </c>
       <c r="J78" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr"/>
@@ -4594,7 +4602,11 @@
           <t>PNG</t>
         </is>
       </c>
-      <c r="F90" s="2" t="inlineStr"/>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>F7;F29</t>
+        </is>
+      </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -4605,10 +4617,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I90" s="2" t="inlineStr"/>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>Hayley Cape / Susan Roberts access - duty-reallocation candidates.</t>
+        </is>
+      </c>
       <c r="J90" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K90" s="2" t="inlineStr"/>
@@ -4725,7 +4741,11 @@
           <t>PNG</t>
         </is>
       </c>
-      <c r="F93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
       <c r="G93" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -4736,10 +4756,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I93" s="2" t="inlineStr"/>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>Proof of Lord’s effectiveness/qualification.</t>
+        </is>
+      </c>
       <c r="J93" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K93" s="2" t="inlineStr"/>
@@ -4766,7 +4790,11 @@
           <t>PAGES</t>
         </is>
       </c>
-      <c r="F94" s="2" t="inlineStr"/>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>F29</t>
+        </is>
+      </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -4777,10 +4805,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I94" s="2" t="inlineStr"/>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>Website ownership - who assumed website duties.</t>
+        </is>
+      </c>
       <c r="J94" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K94" s="2" t="inlineStr"/>
@@ -4967,7 +4999,11 @@
           <t>DOCX</t>
         </is>
       </c>
-      <c r="F99" s="2" t="inlineStr"/>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>L7;F18</t>
+        </is>
+      </c>
       <c r="G99" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -4978,10 +5014,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I99" s="2" t="inlineStr"/>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>Email block/lockout - access cut off.</t>
+        </is>
+      </c>
       <c r="J99" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K99" s="2" t="inlineStr">
@@ -5045,7 +5085,11 @@
           <t>EML</t>
         </is>
       </c>
-      <c r="F101" s="2" t="inlineStr"/>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>F7;F29</t>
+        </is>
+      </c>
       <c r="G101" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -5056,10 +5100,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I101" s="2" t="inlineStr"/>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>Cape Google Business Profile request - marketing duties to Cape.</t>
+        </is>
+      </c>
       <c r="J101" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K101" s="2" t="inlineStr">
@@ -5086,7 +5134,11 @@
           <t>PNG</t>
         </is>
       </c>
-      <c r="F102" s="2" t="inlineStr"/>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
       <c r="G102" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -5097,10 +5149,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I102" s="2" t="inlineStr"/>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>Non-response to Lord.</t>
+        </is>
+      </c>
       <c r="J102" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K102" s="2" t="inlineStr"/>
@@ -5123,7 +5179,11 @@
           <t>EML</t>
         </is>
       </c>
-      <c r="F103" s="2" t="inlineStr"/>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
       <c r="G103" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -5134,10 +5194,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I103" s="2" t="inlineStr"/>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>All-hands / office reassignment / exclusion.</t>
+        </is>
+      </c>
       <c r="J103" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K103" s="2" t="inlineStr">
@@ -5164,7 +5228,11 @@
           <t>PNG</t>
         </is>
       </c>
-      <c r="F104" s="2" t="inlineStr"/>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>F14;F19</t>
+        </is>
+      </c>
       <c r="G104" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -5175,10 +5243,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I104" s="2" t="inlineStr"/>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>Email to T. Phillips re media/reputational exposure (2/25).</t>
+        </is>
+      </c>
       <c r="J104" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K104" s="2" t="inlineStr"/>
@@ -5201,7 +5273,11 @@
           <t>PNG</t>
         </is>
       </c>
-      <c r="F105" s="2" t="inlineStr"/>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>F14;L6</t>
+        </is>
+      </c>
       <c r="G105" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -5212,10 +5288,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I105" s="2" t="inlineStr"/>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>HR/payroll email - payroll issue.</t>
+        </is>
+      </c>
       <c r="J105" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K105" s="2" t="inlineStr"/>
@@ -5283,7 +5363,11 @@
           <t>EML</t>
         </is>
       </c>
-      <c r="F107" s="2" t="inlineStr"/>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
       <c r="G107" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -5294,10 +5378,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I107" s="2" t="inlineStr"/>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>Praise of Lord’s work - rebuts ‘ineffective’ narrative.</t>
+        </is>
+      </c>
       <c r="J107" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K107" s="2" t="inlineStr">
@@ -5361,7 +5449,11 @@
           <t>PNG</t>
         </is>
       </c>
-      <c r="F109" s="2" t="inlineStr"/>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
       <c r="G109" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -5372,10 +5464,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I109" s="2" t="inlineStr"/>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>Monthly meeting w/ Ford - meeting access/cancellations.</t>
+        </is>
+      </c>
       <c r="J109" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K109" s="2" t="inlineStr"/>
@@ -5398,7 +5494,11 @@
           <t>DOCX</t>
         </is>
       </c>
-      <c r="F110" s="2" t="inlineStr"/>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>F24;L5</t>
+        </is>
+      </c>
       <c r="G110" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -5409,10 +5509,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I110" s="2" t="inlineStr"/>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>Email chain raising concerns - protected activity.</t>
+        </is>
+      </c>
       <c r="J110" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K110" s="2" t="inlineStr">
@@ -5443,7 +5547,11 @@
           <t>PNG</t>
         </is>
       </c>
-      <c r="F111" s="2" t="inlineStr"/>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
       <c r="G111" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -5454,10 +5562,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I111" s="2" t="inlineStr"/>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>Lord performing marketing duties (video approval).</t>
+        </is>
+      </c>
       <c r="J111" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K111" s="2" t="inlineStr"/>
@@ -5484,7 +5596,11 @@
           <t>PNG</t>
         </is>
       </c>
-      <c r="F112" s="2" t="inlineStr"/>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
       <c r="G112" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -5495,10 +5611,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I112" s="2" t="inlineStr"/>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>Proof of Lord’s effectiveness/qualification.</t>
+        </is>
+      </c>
       <c r="J112" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K112" s="2" t="inlineStr"/>
@@ -5566,7 +5686,11 @@
           <t>TXT</t>
         </is>
       </c>
-      <c r="F114" s="2" t="inlineStr"/>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>F25;L5</t>
+        </is>
+      </c>
       <c r="G114" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -5577,10 +5701,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I114" s="2" t="inlineStr"/>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>Firearm / safety concerns - protected safety report.</t>
+        </is>
+      </c>
       <c r="J114" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -5689,7 +5817,11 @@
           <t>PNG</t>
         </is>
       </c>
-      <c r="F117" s="2" t="inlineStr"/>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>F19</t>
+        </is>
+      </c>
       <c r="G117" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -5700,10 +5832,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I117" s="2" t="inlineStr"/>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>Request to HR - access/marginalization.</t>
+        </is>
+      </c>
       <c r="J117" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -5730,7 +5866,11 @@
           <t>PDF</t>
         </is>
       </c>
-      <c r="F118" s="2" t="inlineStr"/>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
       <c r="G118" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -5741,10 +5881,14 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="I118" s="2" t="inlineStr"/>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>Lord’s training/certification - qualifications.</t>
+        </is>
+      </c>
       <c r="J118" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr">
@@ -5824,7 +5968,11 @@
           <t>PDF</t>
         </is>
       </c>
-      <c r="F120" s="2" t="inlineStr"/>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
       <c r="G120" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -5835,10 +5983,14 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="I120" s="2" t="inlineStr"/>
+      <c r="I120" s="2" t="inlineStr">
+        <is>
+          <t>Lord’s marketing work product.</t>
+        </is>
+      </c>
       <c r="J120" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K120" s="2" t="inlineStr">
@@ -5869,7 +6021,11 @@
           <t>PDF</t>
         </is>
       </c>
-      <c r="F121" s="2" t="inlineStr"/>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>F4;F5</t>
+        </is>
+      </c>
       <c r="G121" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -5880,10 +6036,14 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="I121" s="2" t="inlineStr"/>
+      <c r="I121" s="2" t="inlineStr">
+        <is>
+          <t>Employment agreement - transfer/comp terms.</t>
+        </is>
+      </c>
       <c r="J121" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K121" s="2" t="inlineStr">
@@ -6135,7 +6295,11 @@
           <t>DOCX</t>
         </is>
       </c>
-      <c r="F127" s="2" t="inlineStr"/>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>F4;F8</t>
+        </is>
+      </c>
       <c r="G127" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -6146,10 +6310,14 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="I127" s="2" t="inlineStr"/>
+      <c r="I127" s="2" t="inlineStr">
+        <is>
+          <t>Marketing Director job description - role/qualifications.</t>
+        </is>
+      </c>
       <c r="J127" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K127" s="2" t="inlineStr">
@@ -6176,7 +6344,11 @@
           <t>PDF</t>
         </is>
       </c>
-      <c r="F128" s="2" t="inlineStr"/>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>F4;F8</t>
+        </is>
+      </c>
       <c r="G128" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -6187,10 +6359,14 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="I128" s="2" t="inlineStr"/>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>Marketing Director job description (HR) - role/qualifications.</t>
+        </is>
+      </c>
       <c r="J128" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K128" s="2" t="inlineStr">
@@ -6336,7 +6512,11 @@
           <t>DOCX</t>
         </is>
       </c>
-      <c r="F132" s="2" t="inlineStr"/>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
       <c r="G132" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -6347,10 +6527,14 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="I132" s="2" t="inlineStr"/>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>Director of Marketing process/duties.</t>
+        </is>
+      </c>
       <c r="J132" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K132" s="2" t="inlineStr">
@@ -6377,7 +6561,11 @@
           <t>DOCX</t>
         </is>
       </c>
-      <c r="F133" s="2" t="inlineStr"/>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
       <c r="G133" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -6388,10 +6576,14 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="I133" s="2" t="inlineStr"/>
+      <c r="I133" s="2" t="inlineStr">
+        <is>
+          <t>Lord’s CV - qualifications (25+ yrs).</t>
+        </is>
+      </c>
       <c r="J133" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K133" s="2" t="inlineStr">
@@ -6418,7 +6610,11 @@
           <t>PDF</t>
         </is>
       </c>
-      <c r="F134" s="2" t="inlineStr"/>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>F4;F5</t>
+        </is>
+      </c>
       <c r="G134" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -6429,10 +6625,14 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="I134" s="2" t="inlineStr"/>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>Salary letter - compensation terms.</t>
+        </is>
+      </c>
       <c r="J134" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K134" s="2" t="inlineStr">
@@ -6549,7 +6749,11 @@
           <t>PDF</t>
         </is>
       </c>
-      <c r="F137" s="2" t="inlineStr"/>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>F3;F4</t>
+        </is>
+      </c>
       <c r="G137" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -6560,10 +6764,14 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="I137" s="2" t="inlineStr"/>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
+          <t>Employment agreement - transfer terms.</t>
+        </is>
+      </c>
       <c r="J137" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K137" s="2" t="inlineStr">
@@ -6766,7 +6974,11 @@
           <t>PDF</t>
         </is>
       </c>
-      <c r="F142" s="2" t="inlineStr"/>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>L3;F13</t>
+        </is>
+      </c>
       <c r="G142" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -6777,10 +6989,14 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="I142" s="2" t="inlineStr"/>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
+          <t>The Dec 2025 disciplinary/verbal warning.</t>
+        </is>
+      </c>
       <c r="J142" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -6803,7 +7019,11 @@
           <t>PDF</t>
         </is>
       </c>
-      <c r="F143" s="2" t="inlineStr"/>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>F3;F4</t>
+        </is>
+      </c>
       <c r="G143" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -6814,10 +7034,14 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="I143" s="2" t="inlineStr"/>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
+          <t>Job change/transfer documentation.</t>
+        </is>
+      </c>
       <c r="J143" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr"/>
@@ -6840,7 +7064,11 @@
           <t>DOCX</t>
         </is>
       </c>
-      <c r="F144" s="2" t="inlineStr"/>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>F4;F19</t>
+        </is>
+      </c>
       <c r="G144" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -6851,10 +7079,14 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="I144" s="2" t="inlineStr"/>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t>Removal of office - marginalization.</t>
+        </is>
+      </c>
       <c r="J144" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -6881,7 +7113,11 @@
           <t>DOCX</t>
         </is>
       </c>
-      <c r="F145" s="2" t="inlineStr"/>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>F6;F19</t>
+        </is>
+      </c>
       <c r="G145" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -6892,10 +7128,14 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="I145" s="2" t="inlineStr"/>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>Lord’s letter to Phillips - reputational/role concerns.</t>
+        </is>
+      </c>
       <c r="J145" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -6967,7 +7207,11 @@
           <t>DOCX</t>
         </is>
       </c>
-      <c r="F147" s="2" t="inlineStr"/>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>F29</t>
+        </is>
+      </c>
       <c r="G147" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -6978,10 +7222,14 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="I147" s="2" t="inlineStr"/>
+      <c r="I147" s="2" t="inlineStr">
+        <is>
+          <t>Susan Roberts agreement - duty-reallocation candidate.</t>
+        </is>
+      </c>
       <c r="J147" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K147" s="2" t="inlineStr"/>
@@ -7168,7 +7416,11 @@
           <t>PDF</t>
         </is>
       </c>
-      <c r="F152" s="2" t="inlineStr"/>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
       <c r="G152" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -7179,10 +7431,14 @@
           <t>Background</t>
         </is>
       </c>
-      <c r="I152" s="2" t="inlineStr"/>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
+          <t>Lord profile/CV - qualifications.</t>
+        </is>
+      </c>
       <c r="J152" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr">
@@ -8012,7 +8268,11 @@
           <t>PNG</t>
         </is>
       </c>
-      <c r="F172" s="2" t="inlineStr"/>
+      <c r="F172" s="2" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
       <c r="G172" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -8023,10 +8283,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I172" s="2" t="inlineStr"/>
+      <c r="I172" s="2" t="inlineStr">
+        <is>
+          <t>Lord’s certification - qualifications.</t>
+        </is>
+      </c>
       <c r="J172" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K172" s="2" t="inlineStr"/>
@@ -8090,7 +8354,11 @@
           <t>PNG</t>
         </is>
       </c>
-      <c r="F174" s="2" t="inlineStr"/>
+      <c r="F174" s="2" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
       <c r="G174" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -8101,10 +8369,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I174" s="2" t="inlineStr"/>
+      <c r="I174" s="2" t="inlineStr">
+        <is>
+          <t>Lord’s marketing work product.</t>
+        </is>
+      </c>
       <c r="J174" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K174" s="2" t="inlineStr"/>
@@ -8127,7 +8399,11 @@
           <t>PNG</t>
         </is>
       </c>
-      <c r="F175" s="2" t="inlineStr"/>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
       <c r="G175" s="3" t="inlineStr">
         <is>
           <t>Supports</t>
@@ -8138,10 +8414,14 @@
           <t>Corroborating</t>
         </is>
       </c>
-      <c r="I175" s="2" t="inlineStr"/>
+      <c r="I175" s="2" t="inlineStr">
+        <is>
+          <t>Lord’s certification - qualifications.</t>
+        </is>
+      </c>
       <c r="J175" s="4" t="inlineStr">
         <is>
-          <t>provisional — review</t>
+          <t>provisional - review</t>
         </is>
       </c>
       <c r="K175" s="2" t="inlineStr"/>

</xml_diff>